<commit_message>
Ship the cedant seed file with only its header
Revision 0005 would otherwise load 25 placeholder names into CIC's database. The seed tests no longer pin a name count, so the client's list can replace the file without a test change.
</commit_message>
<xml_diff>
--- a/db/bootstrap/seed/cedants.xlsx
+++ b/db/bootstrap/seed/cedants.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Cedants" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,11 +413,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A26"/>
+  <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -426,181 +423,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Old Mill Casualty Company</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Bluewater Property &amp; Casualty</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Harbor Casualty Company</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Cardinal Indemnity Company</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Sandhill Mutual Insurance</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Redwood Insurance Exchange</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Copper Valley Specialty Insurance</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Mesa Re</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Evergreen Casualty Company</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Heritage Insurance Exchange</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Tidewater Assurance Group</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Frontier Mutual Insurance</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Willow Bend Property &amp; Casualty</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Twin Rivers Specialty Insurance</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Prairie Property &amp; Casualty</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Riverbend Farm Mutual</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Granite Re</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Stonebridge Farm Mutual</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Highland Assurance Group</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Ironwood General Insurance</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Keystone Specialty Insurance</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Summit Casualty Company</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Silver Creek General Insurance</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Lakeshore Re</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Pinecrest Insurance Exchange</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>